<commit_message>
fix quotation, typo, and colon
</commit_message>
<xml_diff>
--- a/development/processed/airdata/corrected_data_step_2.xlsx
+++ b/development/processed/airdata/corrected_data_step_2.xlsx
@@ -516,7 +516,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Reaching maximum altitude.</t>
+          <t>Reaching maximum altitude...</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cannot switch flight mode. Turn on "Multiple Flight Modes" to enable Atti and Sport Modes.</t>
+          <t>Cannot switch flight mode. Turn on Multiple Flight Modes to enable Atti and Sport Modes.</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Aircraft close to Home Point. "go home" shifts to "landing".</t>
+          <t>Aircraft close to Home Point. go home shifts to landing.</t>
         </is>
       </c>
     </row>

</xml_diff>